<commit_message>
update ni nich 101
</commit_message>
<xml_diff>
--- a/source-data/trading-data.xlsx
+++ b/source-data/trading-data.xlsx
@@ -21646,7 +21646,7 @@
         <v>26.5</v>
       </c>
       <c r="D506" s="3">
-        <v>280</v>
+        <v>350</v>
       </c>
       <c r="E506" s="3">
         <v>1100</v>
@@ -24850,10 +24850,10 @@
         <v>32.5</v>
       </c>
       <c r="D667" s="3">
-        <v>420</v>
+        <v>450</v>
       </c>
       <c r="E667" s="3">
-        <v>1000</v>
+        <v>1250</v>
       </c>
       <c r="F667" s="3">
         <v>4000</v>
@@ -25742,7 +25742,7 @@
         <v>25</v>
       </c>
       <c r="D712" s="3">
-        <v>300</v>
+        <v>350</v>
       </c>
       <c r="E712" s="3">
         <v>700</v>

</xml_diff>

<commit_message>
Update trading data, fix alphabetical ordering, replace zero values with blanks, update image paths, and sync latest spreadsheet changes
</commit_message>
<xml_diff>
--- a/source-data/trading-data.xlsx
+++ b/source-data/trading-data.xlsx
@@ -16083,13 +16083,13 @@
     </dxf>
   </dxfs>
   <tableStyles count="2" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16">
-    <tableStyle name="Pet Wear-style" pivot="0" count="4" xr9:uid="{A5C48195-EEC2-4DCA-85EE-B76662872FC8}">
+    <tableStyle name="Pet Wear-style" pivot="0" count="4" xr9:uid="{65EE2102-1BC9-4F26-9CE3-F450E931A68D}">
       <tableStyleElement type="wholeTable" dxfId="16"/>
       <tableStyleElement type="headerRow" dxfId="15"/>
       <tableStyleElement type="firstRowStripe" dxfId="14"/>
       <tableStyleElement type="secondRowStripe" dxfId="13"/>
     </tableStyle>
-    <tableStyle name="Pets-style" pivot="0" count="4" xr9:uid="{8FA0FFCC-A7A6-4E1F-9ECE-535FC510435C}">
+    <tableStyle name="Pets-style" pivot="0" count="4" xr9:uid="{D96CA825-2139-492E-94AF-1EEDB8536D38}">
       <tableStyleElement type="wholeTable" dxfId="20"/>
       <tableStyleElement type="headerRow" dxfId="19"/>
       <tableStyleElement type="firstRowStripe" dxfId="18"/>
@@ -19427,7 +19427,7 @@
         <v>1700</v>
       </c>
       <c r="D75" s="17">
-        <v>60000</v>
+        <v>6000</v>
       </c>
       <c r="E75" s="17">
         <v>21750</v>

</xml_diff>

<commit_message>
checkpoint: MM2 Nich page implementation
</commit_message>
<xml_diff>
--- a/source-data/trading-data.xlsx
+++ b/source-data/trading-data.xlsx
@@ -5202,7 +5202,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I1008"/>
+  <dimension ref="A1:I1010"/>
   <cols>
     <col min="1" max="1" customWidth="1" width="28"/>
     <col min="2" max="2" customWidth="1" width="42"/>
@@ -5379,13 +5379,13 @@
         <v>1450</v>
       </c>
       <c r="G7">
-        <v>7</v>
+        <v>6.75</v>
       </c>
       <c r="H7">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="I7">
-        <v>128</v>
+        <v>124</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
@@ -5483,13 +5483,13 @@
         <v>23100</v>
       </c>
       <c r="G11">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="H11">
-        <v>532</v>
+        <v>538</v>
       </c>
       <c r="I11">
-        <v>1940</v>
+        <v>1980</v>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
@@ -5665,13 +5665,13 @@
         <v>2520</v>
       </c>
       <c r="G18">
-        <v>20.25</v>
+        <v>21</v>
       </c>
       <c r="H18">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="I18">
-        <v>322</v>
+        <v>340</v>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
@@ -5977,13 +5977,13 @@
         <v>700</v>
       </c>
       <c r="G30">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="H30">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="I30">
-        <v>57</v>
+        <v>70</v>
       </c>
     </row>
     <row r="31" ht="20" customHeight="1">
@@ -6055,7 +6055,7 @@
         <v>4220</v>
       </c>
       <c r="G33">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H33">
         <v>99</v>
@@ -6159,13 +6159,13 @@
         <v>330</v>
       </c>
       <c r="G37">
-        <v>0.98</v>
+        <v>1</v>
       </c>
       <c r="H37">
-        <v>6.86</v>
+        <v>7</v>
       </c>
       <c r="I37">
-        <v>27.8</v>
+        <v>28.45</v>
       </c>
     </row>
     <row r="38" ht="20" customHeight="1">
@@ -6422,10 +6422,10 @@
         <v>167</v>
       </c>
       <c r="H47">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="I47">
-        <v>2000</v>
+        <v>2030</v>
       </c>
     </row>
     <row r="48" ht="20" customHeight="1">
@@ -6549,13 +6549,13 @@
         <v>83400</v>
       </c>
       <c r="G52">
-        <v>920</v>
+        <v>927</v>
       </c>
       <c r="H52">
-        <v>2170</v>
+        <v>2185</v>
       </c>
       <c r="I52">
-        <v>6900</v>
+        <v>6760</v>
       </c>
     </row>
     <row r="53" ht="20" customHeight="1">
@@ -6731,13 +6731,13 @@
         <v>230</v>
       </c>
       <c r="G59">
-        <v>0.75</v>
+        <v>0.77</v>
       </c>
       <c r="H59">
-        <v>4.55</v>
+        <v>4.65</v>
       </c>
       <c r="I59">
-        <v>19.2</v>
+        <v>19.6</v>
       </c>
     </row>
     <row r="60" ht="20" customHeight="1">
@@ -6887,13 +6887,13 @@
         <v>75</v>
       </c>
       <c r="G65">
-        <v>0.17</v>
+        <v>0.18</v>
       </c>
       <c r="H65">
-        <v>1.65</v>
+        <v>1.7</v>
       </c>
       <c r="I65">
-        <v>6.75</v>
+        <v>7</v>
       </c>
     </row>
     <row r="66" ht="20" customHeight="1">
@@ -7121,13 +7121,13 @@
         <v>2440</v>
       </c>
       <c r="G74">
-        <v>12.5</v>
+        <v>13.75</v>
       </c>
       <c r="H74">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="I74">
-        <v>220</v>
+        <v>248</v>
       </c>
     </row>
     <row r="75" ht="20" customHeight="1">
@@ -7173,13 +7173,13 @@
         <v>24120</v>
       </c>
       <c r="G76">
-        <v>148.5</v>
+        <v>198</v>
       </c>
       <c r="H76">
-        <v>590</v>
+        <v>760</v>
       </c>
       <c r="I76">
-        <v>2200</v>
+        <v>2925</v>
       </c>
     </row>
     <row r="77" ht="20" customHeight="1">
@@ -7745,13 +7745,13 @@
         <v>3090</v>
       </c>
       <c r="G98">
-        <v>20</v>
+        <v>20.5</v>
       </c>
       <c r="H98">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="I98">
-        <v>306</v>
+        <v>334</v>
       </c>
     </row>
     <row r="99" ht="20" customHeight="1">
@@ -7797,13 +7797,13 @@
         <v>2640</v>
       </c>
       <c r="G100">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="H100">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I100">
-        <v>227</v>
+        <v>234</v>
       </c>
     </row>
     <row r="101" ht="20" customHeight="1">
@@ -7849,13 +7849,13 @@
         <v>980</v>
       </c>
       <c r="G102">
-        <v>4.25</v>
+        <v>4.5</v>
       </c>
       <c r="H102">
-        <v>20</v>
+        <v>20.5</v>
       </c>
       <c r="I102">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="103" ht="20" customHeight="1">
@@ -7866,13 +7866,13 @@
         <v>/images/pets/Cake Friend.png</v>
       </c>
       <c r="G103">
-        <v>1.02</v>
+        <v>1</v>
       </c>
       <c r="H103">
-        <v>5.95</v>
+        <v>5.85</v>
       </c>
       <c r="I103">
-        <v>24.8</v>
+        <v>24.4</v>
       </c>
     </row>
     <row r="104" ht="20" customHeight="1">
@@ -7976,7 +7976,7 @@
         <v>35</v>
       </c>
       <c r="I107">
-        <v>99</v>
+        <v>105</v>
       </c>
     </row>
     <row r="108" ht="20" customHeight="1">
@@ -8247,13 +8247,13 @@
         <v>645</v>
       </c>
       <c r="G118">
-        <v>2.5</v>
+        <v>4</v>
       </c>
       <c r="H118">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="I118">
-        <v>54</v>
+        <v>78</v>
       </c>
     </row>
     <row r="119" ht="20" customHeight="1">
@@ -8628,10 +8628,10 @@
         <v>5500</v>
       </c>
       <c r="G133">
-        <v>32.5</v>
+        <v>33.5</v>
       </c>
       <c r="H133">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="I133">
         <v>510</v>
@@ -8732,13 +8732,13 @@
         <v>850</v>
       </c>
       <c r="G137">
-        <v>4.25</v>
+        <v>7</v>
       </c>
       <c r="H137">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="I137">
-        <v>83</v>
+        <v>120</v>
       </c>
     </row>
     <row r="138" ht="20" customHeight="1">
@@ -9278,10 +9278,10 @@
         <v>15900</v>
       </c>
       <c r="G158">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="H158">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="I158">
         <v>1210</v>
@@ -9304,13 +9304,13 @@
         <v>14040</v>
       </c>
       <c r="G159">
-        <v>134.5</v>
+        <v>136</v>
       </c>
       <c r="H159">
-        <v>345</v>
+        <v>390</v>
       </c>
       <c r="I159">
-        <v>1360</v>
+        <v>1450</v>
       </c>
     </row>
     <row r="160" ht="20" customHeight="1">
@@ -9356,13 +9356,13 @@
         <v>1250</v>
       </c>
       <c r="G161">
-        <v>5.75</v>
+        <v>6</v>
       </c>
       <c r="H161">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I161">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
     <row r="162" ht="20" customHeight="1">
@@ -9408,7 +9408,7 @@
         <v>9500</v>
       </c>
       <c r="G163">
-        <v>59</v>
+        <v>59.5</v>
       </c>
       <c r="H163">
         <v>198</v>
@@ -9434,13 +9434,13 @@
         <v>780</v>
       </c>
       <c r="G164">
-        <v>3</v>
+        <v>3.25</v>
       </c>
       <c r="H164">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="I164">
-        <v>62</v>
+        <v>66</v>
       </c>
     </row>
     <row r="165" ht="20" customHeight="1">
@@ -9451,13 +9451,13 @@
         <v>/images/pets/Dango Penguins.png</v>
       </c>
       <c r="G165">
-        <v>2.15</v>
+        <v>2.35</v>
       </c>
       <c r="H165">
-        <v>11.5</v>
+        <v>12.5</v>
       </c>
       <c r="I165">
-        <v>48</v>
+        <v>52</v>
       </c>
     </row>
     <row r="166" ht="20" customHeight="1">
@@ -9555,13 +9555,13 @@
         <v>635</v>
       </c>
       <c r="G169">
-        <v>2.75</v>
+        <v>3.75</v>
       </c>
       <c r="H169">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="I169">
-        <v>58</v>
+        <v>74</v>
       </c>
     </row>
     <row r="170" ht="20" customHeight="1">
@@ -9581,13 +9581,13 @@
         <v>880</v>
       </c>
       <c r="G170">
-        <v>4.25</v>
+        <v>5</v>
       </c>
       <c r="H170">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="I170">
-        <v>84</v>
+        <v>92</v>
       </c>
     </row>
     <row r="171" ht="20" customHeight="1">
@@ -9607,13 +9607,13 @@
         <v>10800</v>
       </c>
       <c r="G171">
-        <v>62.5</v>
+        <v>65</v>
       </c>
       <c r="H171">
-        <v>232</v>
+        <v>258</v>
       </c>
       <c r="I171">
-        <v>925</v>
+        <v>1030</v>
       </c>
     </row>
     <row r="172" ht="20" customHeight="1">
@@ -9711,13 +9711,13 @@
         <v>620</v>
       </c>
       <c r="G175">
-        <v>3.25</v>
+        <v>3.5</v>
       </c>
       <c r="H175">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="I175">
-        <v>66</v>
+        <v>70</v>
       </c>
     </row>
     <row r="176" ht="20" customHeight="1">
@@ -10283,13 +10283,13 @@
         <v>580</v>
       </c>
       <c r="G197">
-        <v>2.75</v>
+        <v>2.85</v>
       </c>
       <c r="H197">
-        <v>14</v>
+        <v>14.5</v>
       </c>
       <c r="I197">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="198" ht="20" customHeight="1">
@@ -10554,13 +10554,13 @@
         <v>1000</v>
       </c>
       <c r="G208">
-        <v>1.65</v>
+        <v>1.05</v>
       </c>
       <c r="H208">
-        <v>9.5</v>
+        <v>7.25</v>
       </c>
       <c r="I208">
-        <v>40</v>
+        <v>30</v>
       </c>
     </row>
     <row r="209" ht="20" customHeight="1">
@@ -10580,13 +10580,13 @@
         <v>2900</v>
       </c>
       <c r="G209">
-        <v>17.5</v>
+        <v>27</v>
       </c>
       <c r="H209">
-        <v>73</v>
+        <v>110</v>
       </c>
       <c r="I209">
-        <v>294</v>
+        <v>450</v>
       </c>
     </row>
     <row r="210" ht="20" customHeight="1">
@@ -10710,13 +10710,13 @@
         <v>100</v>
       </c>
       <c r="G214">
-        <v>0.37</v>
+        <v>0.39</v>
       </c>
       <c r="H214">
-        <v>2.65</v>
+        <v>2.75</v>
       </c>
       <c r="I214">
-        <v>11.6</v>
+        <v>12</v>
       </c>
     </row>
     <row r="215" ht="20" customHeight="1">
@@ -10762,13 +10762,13 @@
         <v>90</v>
       </c>
       <c r="G216">
-        <v>0.32</v>
+        <v>0.34</v>
       </c>
       <c r="H216">
-        <v>2.4</v>
+        <v>2.5</v>
       </c>
       <c r="I216">
-        <v>10.5</v>
+        <v>11</v>
       </c>
     </row>
     <row r="217" ht="20" customHeight="1">
@@ -10788,13 +10788,13 @@
         <v>210</v>
       </c>
       <c r="G217">
-        <v>0.88</v>
+        <v>0.9</v>
       </c>
       <c r="H217">
-        <v>5.15</v>
+        <v>5.25</v>
       </c>
       <c r="I217">
-        <v>21.6</v>
+        <v>22</v>
       </c>
     </row>
     <row r="218" ht="20" customHeight="1">
@@ -10814,7 +10814,7 @@
         <v>7700</v>
       </c>
       <c r="G218">
-        <v>108</v>
+        <v>108.5</v>
       </c>
       <c r="H218">
         <v>200</v>
@@ -10840,13 +10840,13 @@
         <v>2000</v>
       </c>
       <c r="G219">
-        <v>17</v>
+        <v>17.5</v>
       </c>
       <c r="H219">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="I219">
-        <v>172</v>
+        <v>174</v>
       </c>
     </row>
     <row r="220" ht="20" customHeight="1">
@@ -11464,10 +11464,10 @@
         <v>17000</v>
       </c>
       <c r="G243">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="H243">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="I243">
         <v>1400</v>
@@ -11516,13 +11516,13 @@
         <v>360</v>
       </c>
       <c r="G245">
-        <v>1.35</v>
+        <v>1.75</v>
       </c>
       <c r="H245">
-        <v>8.5</v>
+        <v>10</v>
       </c>
       <c r="I245">
-        <v>36</v>
+        <v>42</v>
       </c>
     </row>
     <row r="246" ht="20" customHeight="1">
@@ -11542,13 +11542,13 @@
         <v>2600</v>
       </c>
       <c r="G246">
-        <v>14</v>
+        <v>14.75</v>
       </c>
       <c r="H246">
-        <v>59.5</v>
+        <v>63</v>
       </c>
       <c r="I246">
-        <v>240</v>
+        <v>256</v>
       </c>
     </row>
     <row r="247" ht="20" customHeight="1">
@@ -11568,13 +11568,13 @@
         <v>5500</v>
       </c>
       <c r="G247">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="H247">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="I247">
-        <v>620</v>
+        <v>590</v>
       </c>
     </row>
     <row r="248" ht="20" customHeight="1">
@@ -11646,13 +11646,13 @@
         <v>70</v>
       </c>
       <c r="G250">
-        <v>0.18</v>
+        <v>0.17</v>
       </c>
       <c r="H250">
-        <v>1.7</v>
+        <v>1.65</v>
       </c>
       <c r="I250">
-        <v>7</v>
+        <v>6.75</v>
       </c>
     </row>
     <row r="251" ht="20" customHeight="1">
@@ -11672,13 +11672,13 @@
         <v>260</v>
       </c>
       <c r="G251">
-        <v>0.88</v>
+        <v>0.9</v>
       </c>
       <c r="H251">
-        <v>5.2</v>
+        <v>5.3</v>
       </c>
       <c r="I251">
-        <v>21.8</v>
+        <v>22.2</v>
       </c>
     </row>
     <row r="252" ht="20" customHeight="1">
@@ -11897,13 +11897,13 @@
         <v>285</v>
       </c>
       <c r="G260">
-        <v>1.03</v>
+        <v>1.55</v>
       </c>
       <c r="H260">
-        <v>6</v>
+        <v>8.6</v>
       </c>
       <c r="I260">
-        <v>25</v>
+        <v>35.4</v>
       </c>
     </row>
     <row r="261" ht="20" customHeight="1">
@@ -11920,13 +11920,13 @@
         <v>80</v>
       </c>
       <c r="G261">
-        <v>0.17</v>
+        <v>0.18</v>
       </c>
       <c r="H261">
-        <v>1.65</v>
+        <v>1.7</v>
       </c>
       <c r="I261">
-        <v>6.75</v>
+        <v>7</v>
       </c>
     </row>
     <row r="262" ht="20" customHeight="1">
@@ -11946,13 +11946,13 @@
         <v>240</v>
       </c>
       <c r="G262">
-        <v>0.8</v>
+        <v>1.45</v>
       </c>
       <c r="H262">
-        <v>4.75</v>
+        <v>8.1</v>
       </c>
       <c r="I262">
-        <v>20</v>
+        <v>33.4</v>
       </c>
     </row>
     <row r="263" ht="20" customHeight="1">
@@ -12024,13 +12024,13 @@
         <v>1290</v>
       </c>
       <c r="G265">
-        <v>6</v>
+        <v>6.5</v>
       </c>
       <c r="H265">
-        <v>26.5</v>
+        <v>28</v>
       </c>
       <c r="I265">
-        <v>108</v>
+        <v>114</v>
       </c>
     </row>
     <row r="266" ht="20" customHeight="1">
@@ -12102,13 +12102,13 @@
         <v>763</v>
       </c>
       <c r="G268">
-        <v>3.15</v>
+        <v>3.75</v>
       </c>
       <c r="H268">
-        <v>15.5</v>
+        <v>17</v>
       </c>
       <c r="I268">
-        <v>64</v>
+        <v>70</v>
       </c>
     </row>
     <row r="269" ht="20" customHeight="1">
@@ -12128,13 +12128,13 @@
         <v>30000</v>
       </c>
       <c r="G269">
-        <v>194.5</v>
+        <v>220</v>
       </c>
       <c r="H269">
-        <v>750</v>
+        <v>870</v>
       </c>
       <c r="I269">
-        <v>2980</v>
+        <v>3250</v>
       </c>
     </row>
     <row r="270" ht="20" customHeight="1">
@@ -12318,13 +12318,13 @@
         <v>34000</v>
       </c>
       <c r="G277">
-        <v>459</v>
+        <v>462</v>
       </c>
       <c r="H277">
-        <v>915</v>
+        <v>920</v>
       </c>
       <c r="I277">
-        <v>3000</v>
+        <v>3075</v>
       </c>
     </row>
     <row r="278" ht="20" customHeight="1">
@@ -12370,13 +12370,13 @@
         <v>810</v>
       </c>
       <c r="G279">
-        <v>7.75</v>
+        <v>5.5</v>
       </c>
       <c r="H279">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="I279">
-        <v>148</v>
+        <v>104</v>
       </c>
     </row>
     <row r="280" ht="20" customHeight="1">
@@ -12445,13 +12445,13 @@
         <v>525</v>
       </c>
       <c r="G282">
-        <v>1.85</v>
+        <v>2</v>
       </c>
       <c r="H282">
-        <v>10.5</v>
+        <v>11</v>
       </c>
       <c r="I282">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="283" ht="20" customHeight="1">
@@ -12471,13 +12471,13 @@
         <v>740</v>
       </c>
       <c r="G283">
-        <v>3</v>
+        <v>3.75</v>
       </c>
       <c r="H283">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="I283">
-        <v>62</v>
+        <v>70</v>
       </c>
     </row>
     <row r="284" ht="20" customHeight="1">
@@ -12543,13 +12543,13 @@
         <v>1440</v>
       </c>
       <c r="G286">
-        <v>6.5</v>
+        <v>7</v>
       </c>
       <c r="H286">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="I286">
-        <v>120</v>
+        <v>130</v>
       </c>
     </row>
     <row r="287" ht="20" customHeight="1">
@@ -13219,13 +13219,13 @@
         <v>4300</v>
       </c>
       <c r="G312">
-        <v>23.25</v>
+        <v>29</v>
       </c>
       <c r="H312">
-        <v>93</v>
+        <v>116</v>
       </c>
       <c r="I312">
-        <v>370</v>
+        <v>460</v>
       </c>
     </row>
     <row r="313" ht="20" customHeight="1">
@@ -13404,10 +13404,10 @@
         <v>119</v>
       </c>
       <c r="H319">
-        <v>434</v>
+        <v>463</v>
       </c>
       <c r="I319">
-        <v>1750</v>
+        <v>1850</v>
       </c>
     </row>
     <row r="320" ht="20" customHeight="1">
@@ -13531,13 +13531,13 @@
         <v>870</v>
       </c>
       <c r="G324">
-        <v>5</v>
+        <v>5.5</v>
       </c>
       <c r="H324">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I324">
-        <v>92</v>
+        <v>100</v>
       </c>
     </row>
     <row r="325" ht="20" customHeight="1">
@@ -13791,13 +13791,13 @@
         <v>160</v>
       </c>
       <c r="G334">
-        <v>0.51</v>
+        <v>0.75</v>
       </c>
       <c r="H334">
-        <v>3.35</v>
+        <v>4.55</v>
       </c>
       <c r="I334">
-        <v>14.4</v>
+        <v>19.2</v>
       </c>
     </row>
     <row r="335" ht="20" customHeight="1">
@@ -13817,7 +13817,7 @@
         <v>12000</v>
       </c>
       <c r="G335">
-        <v>66.75</v>
+        <v>67.25</v>
       </c>
       <c r="H335">
         <v>250</v>
@@ -13869,13 +13869,13 @@
         <v>1080</v>
       </c>
       <c r="G337">
-        <v>7.5</v>
+        <v>8.75</v>
       </c>
       <c r="H337">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="I337">
-        <v>140</v>
+        <v>156</v>
       </c>
     </row>
     <row r="338" ht="20" customHeight="1">
@@ -13973,13 +13973,13 @@
         <v>960</v>
       </c>
       <c r="G341">
-        <v>6.25</v>
+        <v>5</v>
       </c>
       <c r="H341">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="I341">
-        <v>124</v>
+        <v>96</v>
       </c>
     </row>
     <row r="342" ht="20" customHeight="1">
@@ -14311,13 +14311,13 @@
         <v>480</v>
       </c>
       <c r="G354">
-        <v>1.75</v>
+        <v>3.25</v>
       </c>
       <c r="H354">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="I354">
-        <v>42</v>
+        <v>66</v>
       </c>
     </row>
     <row r="355" ht="20" customHeight="1">
@@ -14363,13 +14363,13 @@
         <v>400</v>
       </c>
       <c r="G356">
-        <v>1.45</v>
+        <v>1.8</v>
       </c>
       <c r="H356">
-        <v>8.1</v>
+        <v>9.85</v>
       </c>
       <c r="I356">
-        <v>33.4</v>
+        <v>40.4</v>
       </c>
     </row>
     <row r="357" ht="20" customHeight="1">
@@ -14389,13 +14389,13 @@
         <v>80</v>
       </c>
       <c r="G357">
-        <v>0.18</v>
+        <v>0.17</v>
       </c>
       <c r="H357">
-        <v>1.7</v>
+        <v>1.65</v>
       </c>
       <c r="I357">
-        <v>7</v>
+        <v>6.75</v>
       </c>
     </row>
     <row r="358" ht="20" customHeight="1">
@@ -14571,13 +14571,13 @@
         <v>1750</v>
       </c>
       <c r="G364">
-        <v>9.5</v>
+        <v>9</v>
       </c>
       <c r="H364">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="I364">
-        <v>166</v>
+        <v>158</v>
       </c>
     </row>
     <row r="365" ht="20" customHeight="1">
@@ -14649,13 +14649,13 @@
         <v>7000</v>
       </c>
       <c r="G367">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="H367">
-        <v>186</v>
+        <v>215</v>
       </c>
       <c r="I367">
-        <v>740</v>
+        <v>855</v>
       </c>
     </row>
     <row r="368" ht="20" customHeight="1">
@@ -14675,13 +14675,13 @@
         <v>2050</v>
       </c>
       <c r="G368">
-        <v>9.75</v>
+        <v>9.5</v>
       </c>
       <c r="H368">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="I368">
-        <v>168</v>
+        <v>160</v>
       </c>
     </row>
     <row r="369" ht="20" customHeight="1">
@@ -14727,13 +14727,13 @@
         <v>980</v>
       </c>
       <c r="G370">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="H370">
-        <v>27</v>
+        <v>39</v>
       </c>
       <c r="I370">
-        <v>110</v>
+        <v>158</v>
       </c>
     </row>
     <row r="371" ht="20" customHeight="1">
@@ -14863,7 +14863,7 @@
         <v>39</v>
       </c>
       <c r="I375">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="376" ht="20" customHeight="1">
@@ -14909,13 +14909,13 @@
         <v>200</v>
       </c>
       <c r="G377">
-        <v>0.66</v>
+        <v>0.67</v>
       </c>
       <c r="H377">
-        <v>4.1</v>
+        <v>4.15</v>
       </c>
       <c r="I377">
-        <v>17.4</v>
+        <v>17.6</v>
       </c>
     </row>
     <row r="378" ht="20" customHeight="1">
@@ -14935,13 +14935,13 @@
         <v>280</v>
       </c>
       <c r="G378">
-        <v>3.75</v>
+        <v>2.75</v>
       </c>
       <c r="H378">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="I378">
-        <v>74</v>
+        <v>60</v>
       </c>
     </row>
     <row r="379" ht="20" customHeight="1">
@@ -15299,13 +15299,13 @@
         <v>500</v>
       </c>
       <c r="G392">
-        <v>2.15</v>
+        <v>2.5</v>
       </c>
       <c r="H392">
-        <v>11.5</v>
+        <v>12.5</v>
       </c>
       <c r="I392">
-        <v>48</v>
+        <v>52</v>
       </c>
     </row>
     <row r="393" ht="20" customHeight="1">
@@ -15429,13 +15429,13 @@
         <v>480</v>
       </c>
       <c r="G397">
-        <v>1.75</v>
+        <v>1.85</v>
       </c>
       <c r="H397">
-        <v>10</v>
+        <v>10.5</v>
       </c>
       <c r="I397">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="398" ht="20" customHeight="1">
@@ -15455,13 +15455,13 @@
         <v>1150</v>
       </c>
       <c r="G398">
-        <v>5.5</v>
+        <v>5.25</v>
       </c>
       <c r="H398">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="I398">
-        <v>100</v>
+        <v>96</v>
       </c>
     </row>
     <row r="399" ht="20" customHeight="1">
@@ -15481,13 +15481,13 @@
         <v>320</v>
       </c>
       <c r="G399">
-        <v>0.97</v>
+        <v>1.15</v>
       </c>
       <c r="H399">
-        <v>6.79</v>
+        <v>7.5</v>
       </c>
       <c r="I399">
-        <v>27.5</v>
+        <v>31</v>
       </c>
     </row>
     <row r="400" ht="20" customHeight="1">
@@ -15510,10 +15510,10 @@
         <v>2</v>
       </c>
       <c r="H400">
-        <v>10.5</v>
+        <v>11</v>
       </c>
       <c r="I400">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="401" ht="20" customHeight="1">
@@ -16321,13 +16321,13 @@
         <v>1520</v>
       </c>
       <c r="G432">
-        <v>15.5</v>
+        <v>18</v>
       </c>
       <c r="H432">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="I432">
-        <v>260</v>
+        <v>300</v>
       </c>
     </row>
     <row r="433" ht="20" customHeight="1">
@@ -16500,13 +16500,13 @@
         <v>850</v>
       </c>
       <c r="G439">
-        <v>4.75</v>
+        <v>5.5</v>
       </c>
       <c r="H439">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="I439">
-        <v>90</v>
+        <v>102</v>
       </c>
     </row>
     <row r="440" ht="20" customHeight="1">
@@ -16780,13 +16780,13 @@
         <v>6520</v>
       </c>
       <c r="G450">
-        <v>34.5</v>
+        <v>37</v>
       </c>
       <c r="H450">
-        <v>138</v>
+        <v>147</v>
       </c>
       <c r="I450">
-        <v>550</v>
+        <v>590</v>
       </c>
     </row>
     <row r="451" ht="20" customHeight="1">
@@ -16832,13 +16832,13 @@
         <v>360</v>
       </c>
       <c r="G452">
-        <v>1.3</v>
+        <v>1.5</v>
       </c>
       <c r="H452">
-        <v>8.5</v>
+        <v>9</v>
       </c>
       <c r="I452">
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
     <row r="453" ht="20" customHeight="1">
@@ -16858,13 +16858,13 @@
         <v>3250</v>
       </c>
       <c r="G453">
-        <v>16.75</v>
+        <v>16.25</v>
       </c>
       <c r="H453">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="I453">
-        <v>300</v>
+        <v>292</v>
       </c>
     </row>
     <row r="454" ht="20" customHeight="1">
@@ -17481,13 +17481,13 @@
         <v>65</v>
       </c>
       <c r="G478">
-        <v>0.11</v>
+        <v>0.12</v>
       </c>
       <c r="H478">
-        <v>1.55</v>
+        <v>1.6</v>
       </c>
       <c r="I478">
-        <v>5.25</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="479" ht="20" customHeight="1">
@@ -17744,10 +17744,10 @@
         <v>105</v>
       </c>
       <c r="H488">
-        <v>375</v>
+        <v>401</v>
       </c>
       <c r="I488">
-        <v>1500</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="489" ht="20" customHeight="1">
@@ -17868,10 +17868,10 @@
         <v>24300</v>
       </c>
       <c r="G493">
-        <v>242</v>
+        <v>243.5</v>
       </c>
       <c r="H493">
-        <v>601</v>
+        <v>603</v>
       </c>
       <c r="I493">
         <v>1860</v>
@@ -18050,10 +18050,10 @@
         <v>12300</v>
       </c>
       <c r="G500">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="H500">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="I500">
         <v>1025</v>
@@ -18284,13 +18284,13 @@
         <v>2800</v>
       </c>
       <c r="G509">
-        <v>26.75</v>
+        <v>27</v>
       </c>
       <c r="H509">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="I509">
-        <v>380</v>
+        <v>400</v>
       </c>
     </row>
     <row r="510" ht="20" customHeight="1">
@@ -18370,13 +18370,13 @@
         <v>1320</v>
       </c>
       <c r="G513">
-        <v>8.25</v>
+        <v>9.25</v>
       </c>
       <c r="H513">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="I513">
-        <v>144</v>
+        <v>160</v>
       </c>
     </row>
     <row r="514" ht="20" customHeight="1">
@@ -18604,13 +18604,13 @@
         <v>3000</v>
       </c>
       <c r="G522">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="H522">
-        <v>71</v>
+        <v>99</v>
       </c>
       <c r="I522">
-        <v>286</v>
+        <v>400</v>
       </c>
     </row>
     <row r="523" ht="20" customHeight="1">
@@ -18884,13 +18884,13 @@
         <v>230</v>
       </c>
       <c r="G533">
-        <v>0.72</v>
+        <v>0.73</v>
       </c>
       <c r="H533">
-        <v>4.4</v>
+        <v>4.45</v>
       </c>
       <c r="I533">
-        <v>18.6</v>
+        <v>18.8</v>
       </c>
     </row>
     <row r="534" ht="20" customHeight="1">
@@ -19248,13 +19248,13 @@
         <v>70</v>
       </c>
       <c r="G547">
-        <v>0.17</v>
+        <v>0.18</v>
       </c>
       <c r="H547">
-        <v>1.65</v>
+        <v>1.7</v>
       </c>
       <c r="I547">
-        <v>6.75</v>
+        <v>7</v>
       </c>
     </row>
     <row r="548" ht="20" customHeight="1">
@@ -19274,13 +19274,13 @@
         <v>420</v>
       </c>
       <c r="G548">
-        <v>3</v>
+        <v>3.25</v>
       </c>
       <c r="H548">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="I548">
-        <v>62</v>
+        <v>66</v>
       </c>
     </row>
     <row r="549" ht="20" customHeight="1">
@@ -19326,13 +19326,13 @@
         <v>440</v>
       </c>
       <c r="G550">
-        <v>1.55</v>
+        <v>2</v>
       </c>
       <c r="H550">
-        <v>9.25</v>
+        <v>11</v>
       </c>
       <c r="I550">
-        <v>39</v>
+        <v>46</v>
       </c>
     </row>
     <row r="551" ht="20" customHeight="1">
@@ -19690,13 +19690,13 @@
         <v>2730</v>
       </c>
       <c r="G564">
-        <v>11.5</v>
+        <v>7.5</v>
       </c>
       <c r="H564">
-        <v>51</v>
+        <v>34</v>
       </c>
       <c r="I564">
-        <v>210</v>
+        <v>142</v>
       </c>
     </row>
     <row r="565" ht="20" customHeight="1">
@@ -19794,13 +19794,13 @@
         <v>280</v>
       </c>
       <c r="G568">
-        <v>0.99</v>
+        <v>0.96</v>
       </c>
       <c r="H568">
-        <v>5.75</v>
+        <v>5.6</v>
       </c>
       <c r="I568">
-        <v>24</v>
+        <v>23.4</v>
       </c>
     </row>
     <row r="569" ht="20" customHeight="1">
@@ -20282,13 +20282,13 @@
         <v>640</v>
       </c>
       <c r="G587">
-        <v>2.5</v>
+        <v>2.75</v>
       </c>
       <c r="H587">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I587">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="588" ht="20" customHeight="1">
@@ -20386,13 +20386,13 @@
         <v>2300</v>
       </c>
       <c r="G591">
-        <v>11.25</v>
+        <v>15</v>
       </c>
       <c r="H591">
-        <v>49</v>
+        <v>64</v>
       </c>
       <c r="I591">
-        <v>200</v>
+        <v>260</v>
       </c>
     </row>
     <row r="592" ht="20" customHeight="1">
@@ -20695,13 +20695,13 @@
         <v>300</v>
       </c>
       <c r="G603">
-        <v>0.97</v>
+        <v>1.05</v>
       </c>
       <c r="H603">
-        <v>6.79</v>
+        <v>7.25</v>
       </c>
       <c r="I603">
-        <v>27.5</v>
+        <v>30</v>
       </c>
     </row>
     <row r="604" ht="20" customHeight="1">
@@ -21085,13 +21085,13 @@
         <v>37000</v>
       </c>
       <c r="G618">
-        <v>672</v>
+        <v>675</v>
       </c>
       <c r="H618">
-        <v>1343</v>
+        <v>1348</v>
       </c>
       <c r="I618">
-        <v>3380</v>
+        <v>3485</v>
       </c>
     </row>
     <row r="619" ht="20" customHeight="1">
@@ -21501,13 +21501,13 @@
         <v>10500</v>
       </c>
       <c r="G634">
-        <v>54</v>
+        <v>23</v>
       </c>
       <c r="H634">
-        <v>225</v>
+        <v>83</v>
       </c>
       <c r="I634">
-        <v>908</v>
+        <v>300</v>
       </c>
     </row>
     <row r="635" ht="20" customHeight="1">
@@ -21579,13 +21579,13 @@
         <v>360</v>
       </c>
       <c r="G637">
-        <v>1.35</v>
+        <v>2.25</v>
       </c>
       <c r="H637">
-        <v>8.5</v>
+        <v>12</v>
       </c>
       <c r="I637">
-        <v>36</v>
+        <v>50</v>
       </c>
     </row>
     <row r="638" ht="20" customHeight="1">
@@ -21657,13 +21657,13 @@
         <v>560</v>
       </c>
       <c r="G640">
-        <v>2.25</v>
+        <v>3.85</v>
       </c>
       <c r="H640">
-        <v>12</v>
+        <v>18.5</v>
       </c>
       <c r="I640">
-        <v>50</v>
+        <v>76</v>
       </c>
     </row>
     <row r="641" ht="20" customHeight="1">
@@ -22021,13 +22021,13 @@
         <v>80</v>
       </c>
       <c r="G654">
-        <v>0.18</v>
+        <v>0.17</v>
       </c>
       <c r="H654">
-        <v>1.7</v>
+        <v>1.65</v>
       </c>
       <c r="I654">
-        <v>7</v>
+        <v>6.75</v>
       </c>
     </row>
     <row r="655" ht="20" customHeight="1">
@@ -22411,13 +22411,13 @@
         <v>980</v>
       </c>
       <c r="G669">
-        <v>4.5</v>
+        <v>5.5</v>
       </c>
       <c r="H669">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="I669">
-        <v>86</v>
+        <v>100</v>
       </c>
     </row>
     <row r="670" ht="20" customHeight="1">
@@ -22437,10 +22437,10 @@
         <v>4800</v>
       </c>
       <c r="G670">
-        <v>33.5</v>
+        <v>34.5</v>
       </c>
       <c r="H670">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="I670">
         <v>428</v>
@@ -22567,13 +22567,13 @@
         <v>1655</v>
       </c>
       <c r="G675">
-        <v>9.5</v>
+        <v>12.5</v>
       </c>
       <c r="H675">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="I675">
-        <v>170</v>
+        <v>220</v>
       </c>
     </row>
     <row r="676" ht="20" customHeight="1">
@@ -23217,13 +23217,13 @@
         <v>2000</v>
       </c>
       <c r="G700">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="H700">
-        <v>53</v>
+        <v>75</v>
       </c>
       <c r="I700">
-        <v>216</v>
+        <v>310</v>
       </c>
     </row>
     <row r="701" ht="20" customHeight="1">
@@ -23269,13 +23269,13 @@
         <v>6500</v>
       </c>
       <c r="G702">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="H702">
-        <v>155</v>
+        <v>110</v>
       </c>
       <c r="I702">
-        <v>630</v>
+        <v>450</v>
       </c>
     </row>
     <row r="703" ht="20" customHeight="1">
@@ -23529,13 +23529,13 @@
         <v>5100</v>
       </c>
       <c r="G712">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="H712">
-        <v>83</v>
+        <v>60</v>
       </c>
       <c r="I712">
-        <v>340</v>
+        <v>250</v>
       </c>
     </row>
     <row r="713" ht="20" customHeight="1">
@@ -23607,13 +23607,13 @@
         <v>1500</v>
       </c>
       <c r="G715">
-        <v>25.25</v>
+        <v>25.5</v>
       </c>
       <c r="H715">
         <v>51.5</v>
       </c>
       <c r="I715">
-        <v>125</v>
+        <v>123</v>
       </c>
     </row>
     <row r="716" ht="20" customHeight="1">
@@ -23702,13 +23702,13 @@
         <v>9500</v>
       </c>
       <c r="G719">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="H719">
-        <v>210</v>
+        <v>252</v>
       </c>
       <c r="I719">
-        <v>828</v>
+        <v>999</v>
       </c>
     </row>
     <row r="720" ht="20" customHeight="1">
@@ -23806,13 +23806,13 @@
         <v>1700</v>
       </c>
       <c r="G723">
-        <v>9.5</v>
+        <v>12</v>
       </c>
       <c r="H723">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="I723">
-        <v>164</v>
+        <v>200</v>
       </c>
     </row>
     <row r="724" ht="20" customHeight="1">
@@ -23884,13 +23884,13 @@
         <v>1600</v>
       </c>
       <c r="G726">
-        <v>7.5</v>
+        <v>13.5</v>
       </c>
       <c r="H726">
-        <v>33</v>
+        <v>57</v>
       </c>
       <c r="I726">
-        <v>136</v>
+        <v>232</v>
       </c>
     </row>
     <row r="727" ht="20" customHeight="1">
@@ -23962,13 +23962,13 @@
         <v>330</v>
       </c>
       <c r="G729">
-        <v>3.5</v>
+        <v>1.85</v>
       </c>
       <c r="H729">
-        <v>17</v>
+        <v>10.5</v>
       </c>
       <c r="I729">
-        <v>72</v>
+        <v>44</v>
       </c>
     </row>
     <row r="730" ht="20" customHeight="1">
@@ -24248,13 +24248,13 @@
         <v>3500</v>
       </c>
       <c r="G740">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="H740">
-        <v>82</v>
+        <v>97</v>
       </c>
       <c r="I740">
-        <v>326</v>
+        <v>385</v>
       </c>
     </row>
     <row r="741" ht="20" customHeight="1">
@@ -24326,13 +24326,13 @@
         <v>290</v>
       </c>
       <c r="G743">
-        <v>0.99</v>
+        <v>0.96</v>
       </c>
       <c r="H743">
-        <v>5.75</v>
+        <v>5.6</v>
       </c>
       <c r="I743">
-        <v>24</v>
+        <v>23.4</v>
       </c>
     </row>
     <row r="744" ht="20" customHeight="1">
@@ -24430,13 +24430,13 @@
         <v>2800</v>
       </c>
       <c r="G747">
-        <v>13.75</v>
+        <v>14.25</v>
       </c>
       <c r="H747">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="I747">
-        <v>240</v>
+        <v>252</v>
       </c>
     </row>
     <row r="748" ht="20" customHeight="1">
@@ -24586,13 +24586,13 @@
         <v>520</v>
       </c>
       <c r="G753">
-        <v>2.75</v>
+        <v>2.15</v>
       </c>
       <c r="H753">
-        <v>14</v>
+        <v>11.5</v>
       </c>
       <c r="I753">
-        <v>58</v>
+        <v>48</v>
       </c>
     </row>
     <row r="754" ht="20" customHeight="1">
@@ -24655,13 +24655,13 @@
         <v>/images/pets/Wooly Rhino.png</v>
       </c>
       <c r="G756">
-        <v>0.67</v>
+        <v>1.35</v>
       </c>
       <c r="H756">
-        <v>4.15</v>
+        <v>7.6</v>
       </c>
       <c r="I756">
-        <v>17.6</v>
+        <v>31.4</v>
       </c>
     </row>
     <row r="757" ht="20" customHeight="1">
@@ -24817,7 +24817,7 @@
         <v>7.25</v>
       </c>
       <c r="I762">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="763" ht="20" customHeight="1">
@@ -24915,13 +24915,13 @@
         <v>1920</v>
       </c>
       <c r="G766">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H766">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="I766">
-        <v>188</v>
+        <v>204</v>
       </c>
     </row>
     <row r="767" ht="20" customHeight="1">
@@ -24967,13 +24967,13 @@
         <v>300</v>
       </c>
       <c r="G768">
-        <v>1.05</v>
+        <v>1.73</v>
       </c>
       <c r="H768">
-        <v>6.1</v>
+        <v>9.5</v>
       </c>
       <c r="I768">
-        <v>25.4</v>
+        <v>39</v>
       </c>
     </row>
     <row r="769" ht="20" customHeight="1"/>
@@ -25223,18 +25223,52 @@
         <v>/images/pets/Chihuahua.png</v>
       </c>
       <c r="G1008">
-        <v>1.33</v>
+        <v>0.51</v>
       </c>
       <c r="H1008">
-        <v>7.5</v>
+        <v>3.35</v>
       </c>
       <c r="I1008">
-        <v>31</v>
+        <v>14.4</v>
+      </c>
+    </row>
+    <row r="1009">
+      <c r="A1009" t="str">
+        <v>Kiwi Kiwi</v>
+      </c>
+      <c r="B1009" t="str">
+        <v>/images/pets/Kiwi Kiwi.png</v>
+      </c>
+      <c r="G1009">
+        <v>3</v>
+      </c>
+      <c r="H1009">
+        <v>15</v>
+      </c>
+      <c r="I1009">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="1010">
+      <c r="A1010" t="str">
+        <v>Strawberry Tortle</v>
+      </c>
+      <c r="B1010" t="str">
+        <v>/images/pets/Strawberry Tortle.png</v>
+      </c>
+      <c r="G1010">
+        <v>29</v>
+      </c>
+      <c r="H1010">
+        <v>125</v>
+      </c>
+      <c r="I1010">
+        <v>515</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I1008"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I1010"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -26897,7 +26931,7 @@
         <v>/images/pets/Buzzing Honeypot Hat.png</v>
       </c>
       <c r="F117">
-        <v>190</v>
+        <v>140</v>
       </c>
     </row>
     <row r="118" ht="20" customHeight="1">
@@ -31538,7 +31572,7 @@
         <v>/images/pets/Hive Backpack.png</v>
       </c>
       <c r="F450">
-        <v>90</v>
+        <v>67</v>
       </c>
     </row>
     <row r="451" ht="20" customHeight="1">
@@ -33612,7 +33646,7 @@
         <v>/images/pets/Panda Cap.png</v>
       </c>
       <c r="F599">
-        <v>1100</v>
+        <v>800</v>
       </c>
     </row>
     <row r="600" ht="20" customHeight="1">
@@ -34429,7 +34463,7 @@
         <v>/images/pets/Queen Bee Slippers.png</v>
       </c>
       <c r="F658">
-        <v>85</v>
+        <v>68</v>
       </c>
     </row>
     <row r="659" ht="20" customHeight="1">
@@ -36450,7 +36484,7 @@
         <v>860</v>
       </c>
       <c r="F803">
-        <v>180</v>
+        <v>165</v>
       </c>
     </row>
     <row r="804" ht="20" customHeight="1">
@@ -36632,7 +36666,7 @@
         <v>940</v>
       </c>
       <c r="F816">
-        <v>190</v>
+        <v>180</v>
       </c>
     </row>
     <row r="817" ht="20" customHeight="1">
@@ -36660,7 +36694,7 @@
         <v>970</v>
       </c>
       <c r="F818">
-        <v>140</v>
+        <v>120</v>
       </c>
     </row>
     <row r="819" ht="20" customHeight="1">
@@ -40563,7 +40597,7 @@
         <v>3445</v>
       </c>
       <c r="D96">
-        <v>345</v>
+        <v>255</v>
       </c>
     </row>
     <row r="97" ht="20" customHeight="1">
@@ -45996,7 +46030,7 @@
         <v>22500</v>
       </c>
       <c r="D510">
-        <v>1930</v>
+        <v>1900</v>
       </c>
     </row>
     <row r="511" ht="20" customHeight="1">
@@ -52822,7 +52856,7 @@
         <v>60</v>
       </c>
       <c r="D23">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1">

</xml_diff>